<commit_message>
Updating examples excel file for "Akorn" SCF 2011-2013. So far 001e is identifying revisions.
</commit_message>
<xml_diff>
--- a/Examples.xlsx
+++ b/Examples.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnpeterson\Git\SCF-Audit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7C1BC62-8D3A-4203-9797-8B5DF9EB890A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C0367CA-097F-489A-8949-E32EB5427B97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-36630" yWindow="6990" windowWidth="23160" windowHeight="15285" activeTab="1" xr2:uid="{D2D55026-8DB7-480C-B7BB-7094D4DE5357}"/>
+    <workbookView xWindow="-56190" yWindow="4260" windowWidth="31830" windowHeight="15930" activeTab="1" xr2:uid="{D2D55026-8DB7-480C-B7BB-7094D4DE5357}"/>
   </bookViews>
   <sheets>
     <sheet name="Walmart Filings" sheetId="3" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="58">
   <si>
     <t>XBRL Tag</t>
   </si>
@@ -193,6 +193,24 @@
   </si>
   <si>
     <t>Change in Trade Accounts Payable</t>
+  </si>
+  <si>
+    <t>*Per 2012 10-K: "Capital expenditures that were accrued but not paid"</t>
+  </si>
+  <si>
+    <t>Akorn Fiscal Year 2012 10-K Statement of Cash Flows</t>
+  </si>
+  <si>
+    <t>End Date = 12/31/2012</t>
+  </si>
+  <si>
+    <t>Akorn Fiscal Year 2013</t>
+  </si>
+  <si>
+    <t>End Date = 12/31/2013</t>
+  </si>
+  <si>
+    <t>*Change of XBRL tags in CFO but actual reclass between line items</t>
   </si>
 </sst>
 </file>
@@ -1536,7 +1554,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54BF230C-2F7D-4629-8124-2990C43312C0}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="50" bestFit="1" customWidth="1"/>
@@ -1546,7 +1564,7 @@
     <col min="5" max="5" width="10.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>49</v>
       </c>
@@ -1555,12 +1573,12 @@
       <c r="D1" s="8"/>
       <c r="E1" s="8"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1577,7 +1595,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>51</v>
       </c>
@@ -1592,7 +1610,7 @@
         <v>3346</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>39</v>
       </c>
@@ -1612,9 +1630,12 @@
       <c r="F7" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="H7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>50</v>
       </c>
@@ -1629,7 +1650,7 @@
         <v>-3346</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -1650,29 +1671,239 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="15" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
+    <row r="12" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="14" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>11</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B14" t="s">
         <v>17</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C14" s="2">
         <v>117716</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D14" s="2">
         <v>117716</v>
       </c>
-      <c r="E15" s="4">
-        <f>C15-D15</f>
-        <v>0</v>
-      </c>
-      <c r="F15" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+      <c r="E14" s="4">
+        <f>C14-D14</f>
+        <v>0</v>
+      </c>
+      <c r="F14" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="3"/>
+      <c r="H21" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>39</v>
+      </c>
+      <c r="B22" t="s">
+        <v>40</v>
+      </c>
+      <c r="C22" s="2">
+        <v>26244</v>
+      </c>
+      <c r="D22" s="2">
+        <v>26244</v>
+      </c>
+      <c r="E22" s="5">
+        <f>C22-D22</f>
+        <v>0</v>
+      </c>
+      <c r="F22" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="25" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>4</v>
+      </c>
+      <c r="B25" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="2">
+        <v>-75501</v>
+      </c>
+      <c r="D25" s="2">
+        <v>-75501</v>
+      </c>
+      <c r="E25" s="4">
+        <f>C25-D25</f>
+        <v>0</v>
+      </c>
+      <c r="F25" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="28" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>11</v>
+      </c>
+      <c r="B28" t="s">
+        <v>17</v>
+      </c>
+      <c r="C28" s="2">
+        <v>6366</v>
+      </c>
+      <c r="D28" s="2">
+        <v>6366</v>
+      </c>
+      <c r="E28" s="4">
+        <f>C28-D28</f>
+        <v>0</v>
+      </c>
+      <c r="F28" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A30" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B30" s="8"/>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="3"/>
+      <c r="H35" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>39</v>
+      </c>
+      <c r="B36" t="s">
+        <v>40</v>
+      </c>
+      <c r="C36" s="2">
+        <v>57326</v>
+      </c>
+      <c r="D36" s="2">
+        <v>57326</v>
+      </c>
+      <c r="E36" s="5">
+        <f>C36-D36</f>
+        <v>0</v>
+      </c>
+      <c r="F36" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="39" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>4</v>
+      </c>
+      <c r="B39" t="s">
+        <v>16</v>
+      </c>
+      <c r="C39" s="2">
+        <v>-66874</v>
+      </c>
+      <c r="D39" s="2">
+        <v>-66874</v>
+      </c>
+      <c r="E39" s="4">
+        <f>C39-D39</f>
+        <v>0</v>
+      </c>
+      <c r="F39" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="42" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>11</v>
+      </c>
+      <c r="B42" t="s">
+        <v>17</v>
+      </c>
+      <c r="C42" s="2">
+        <v>3118</v>
+      </c>
+      <c r="D42" s="2">
+        <v>3118</v>
+      </c>
+      <c r="E42" s="4">
+        <f>C42-D42</f>
+        <v>0</v>
+      </c>
+      <c r="F42" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Adding 2014 for Akorn where things went off the rails for them and had large restatement. 001e script has correctly identified the all the line-by-line revision though.
</commit_message>
<xml_diff>
--- a/Examples.xlsx
+++ b/Examples.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnpeterson\Git\SCF-Audit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C0367CA-097F-489A-8949-E32EB5427B97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03E6613F-974C-4704-A0A7-6D7DA9E1A192}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-56190" yWindow="4260" windowWidth="31830" windowHeight="15930" activeTab="1" xr2:uid="{D2D55026-8DB7-480C-B7BB-7094D4DE5357}"/>
+    <workbookView xWindow="-49755" yWindow="2985" windowWidth="22980" windowHeight="15930" activeTab="1" xr2:uid="{D2D55026-8DB7-480C-B7BB-7094D4DE5357}"/>
   </bookViews>
   <sheets>
     <sheet name="Walmart Filings" sheetId="3" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="77">
   <si>
     <t>XBRL Tag</t>
   </si>
@@ -211,6 +211,63 @@
   </si>
   <si>
     <t>*Change of XBRL tags in CFO but actual reclass between line items</t>
+  </si>
+  <si>
+    <t>Akorn Fiscal Year 2014</t>
+  </si>
+  <si>
+    <t>End Date = 12/31/2014</t>
+  </si>
+  <si>
+    <t>Depreciation &amp; Amortization</t>
+  </si>
+  <si>
+    <t>Amortization of deferred financing fees</t>
+  </si>
+  <si>
+    <t>Gain from product divestiture</t>
+  </si>
+  <si>
+    <t>Deferred income taxes</t>
+  </si>
+  <si>
+    <t>Excess benefit from stock compensation</t>
+  </si>
+  <si>
+    <t>Change in trade accounts receivable, net</t>
+  </si>
+  <si>
+    <t>Change in inventories, net</t>
+  </si>
+  <si>
+    <t>Change in prepaid expenses and other current assets</t>
+  </si>
+  <si>
+    <t>Change in trade accounts payable</t>
+  </si>
+  <si>
+    <t>Change in accrued expenses and other liabilities</t>
+  </si>
+  <si>
+    <t>Consolidated net income</t>
+  </si>
+  <si>
+    <t>Non-cash stock compensation expense</t>
+  </si>
+  <si>
+    <t>Payments for acquisitions and equity investments</t>
+  </si>
+  <si>
+    <t>Proceeds from disposal of assets</t>
+  </si>
+  <si>
+    <t>Purchases of property, plant, and equipment</t>
+  </si>
+  <si>
+    <t>Excess tax benefits from stock compensation</t>
+  </si>
+  <si>
+    <t>Restatement of rebate reserves in addition to many other 'immaterial errors'</t>
   </si>
 </sst>
 </file>
@@ -1554,14 +1611,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54BF230C-2F7D-4629-8124-2990C43312C0}">
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="50" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="40.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.109375" customWidth="1"/>
     <col min="4" max="4" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -1904,6 +1961,346 @@
       </c>
     </row>
     <row r="43" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A44" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B44" s="8"/>
+      <c r="C44" s="8"/>
+      <c r="D44" s="8"/>
+      <c r="E44" s="8"/>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A45" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A47" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>70</v>
+      </c>
+      <c r="C49" s="2">
+        <v>35345</v>
+      </c>
+      <c r="D49" s="2">
+        <v>13884</v>
+      </c>
+      <c r="E49" s="2">
+        <f>C49-D49</f>
+        <v>21461</v>
+      </c>
+      <c r="G49" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>60</v>
+      </c>
+      <c r="C50" s="2">
+        <v>58538</v>
+      </c>
+      <c r="D50" s="2">
+        <v>57831</v>
+      </c>
+      <c r="E50" s="2">
+        <f t="shared" ref="E50:E65" si="0">C50-D50</f>
+        <v>707</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>61</v>
+      </c>
+      <c r="C51" s="2">
+        <v>12129</v>
+      </c>
+      <c r="D51" s="2">
+        <v>9984</v>
+      </c>
+      <c r="E51" s="2">
+        <f t="shared" si="0"/>
+        <v>2145</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>71</v>
+      </c>
+      <c r="C52" s="2">
+        <v>7542</v>
+      </c>
+      <c r="D52" s="2">
+        <v>7752</v>
+      </c>
+      <c r="E52" s="2">
+        <f t="shared" si="0"/>
+        <v>-210</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>62</v>
+      </c>
+      <c r="C53" s="2">
+        <v>-9807</v>
+      </c>
+      <c r="D53" s="2">
+        <v>-9329</v>
+      </c>
+      <c r="E53" s="2">
+        <f t="shared" si="0"/>
+        <v>-478</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>63</v>
+      </c>
+      <c r="C54" s="2">
+        <v>25293</v>
+      </c>
+      <c r="D54" s="2">
+        <v>-17511</v>
+      </c>
+      <c r="E54" s="2">
+        <f t="shared" si="0"/>
+        <v>42804</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>64</v>
+      </c>
+      <c r="C55" s="2">
+        <v>-38710</v>
+      </c>
+      <c r="D55" s="2">
+        <v>-29517</v>
+      </c>
+      <c r="E55" s="2">
+        <f t="shared" si="0"/>
+        <v>-9193</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>65</v>
+      </c>
+      <c r="C56" s="2">
+        <v>-95470</v>
+      </c>
+      <c r="D56" s="2">
+        <v>-72796</v>
+      </c>
+      <c r="E56" s="2">
+        <f t="shared" si="0"/>
+        <v>-22674</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>66</v>
+      </c>
+      <c r="C57" s="2">
+        <v>-15262</v>
+      </c>
+      <c r="D57" s="2">
+        <v>-19385</v>
+      </c>
+      <c r="E57" s="2">
+        <f t="shared" si="0"/>
+        <v>4123</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>67</v>
+      </c>
+      <c r="C58" s="2">
+        <v>-13180</v>
+      </c>
+      <c r="D58" s="2">
+        <v>30372</v>
+      </c>
+      <c r="E58" s="2">
+        <f t="shared" si="0"/>
+        <v>-43552</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>68</v>
+      </c>
+      <c r="C59" s="2">
+        <v>11024</v>
+      </c>
+      <c r="D59" s="2">
+        <v>13963</v>
+      </c>
+      <c r="E59" s="2">
+        <f t="shared" si="0"/>
+        <v>-2939</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>69</v>
+      </c>
+      <c r="C60" s="2">
+        <v>26249</v>
+      </c>
+      <c r="D60" s="2">
+        <v>27967</v>
+      </c>
+      <c r="E60" s="2">
+        <f t="shared" si="0"/>
+        <v>-1718</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>39</v>
+      </c>
+      <c r="B61" t="s">
+        <v>40</v>
+      </c>
+      <c r="C61" s="2">
+        <v>30918</v>
+      </c>
+      <c r="D61" s="2">
+        <v>40442</v>
+      </c>
+      <c r="E61" s="4">
+        <f t="shared" si="0"/>
+        <v>-9524</v>
+      </c>
+      <c r="F61" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>72</v>
+      </c>
+      <c r="C63" s="2">
+        <v>-987802</v>
+      </c>
+      <c r="D63" s="2">
+        <v>-987428</v>
+      </c>
+      <c r="E63" s="2">
+        <f t="shared" si="0"/>
+        <v>-374</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>73</v>
+      </c>
+      <c r="C64" s="2">
+        <v>-8532</v>
+      </c>
+      <c r="D64" s="2">
+        <v>-8908</v>
+      </c>
+      <c r="E64" s="2">
+        <f t="shared" si="0"/>
+        <v>376</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>74</v>
+      </c>
+      <c r="C65" s="2">
+        <v>-29568</v>
+      </c>
+      <c r="D65" s="2">
+        <v>-29899</v>
+      </c>
+      <c r="E65" s="2">
+        <f t="shared" si="0"/>
+        <v>331</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
+        <v>4</v>
+      </c>
+      <c r="B66" t="s">
+        <v>16</v>
+      </c>
+      <c r="C66" s="2">
+        <v>-966541</v>
+      </c>
+      <c r="D66" s="2">
+        <v>-966874</v>
+      </c>
+      <c r="E66" s="4">
+        <f>C66-D66</f>
+        <v>333</v>
+      </c>
+      <c r="F66" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>75</v>
+      </c>
+      <c r="C68" s="2">
+        <v>38710</v>
+      </c>
+      <c r="D68" s="2">
+        <v>29517</v>
+      </c>
+      <c r="E68" s="2">
+        <f t="shared" ref="E68" si="1">C68-D68</f>
+        <v>9193</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>11</v>
+      </c>
+      <c r="B69" t="s">
+        <v>17</v>
+      </c>
+      <c r="C69" s="2">
+        <v>972308</v>
+      </c>
+      <c r="D69" s="2">
+        <v>963116</v>
+      </c>
+      <c r="E69" s="4">
+        <f>C69-D69</f>
+        <v>9192</v>
+      </c>
+      <c r="F69" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>